<commit_message>
Ajustar lista de cotejo de investigación grupal: 4 columnas de integrantes + 5 criterios
Se reemplaza la columna única "Integrantes" por 4 columnas separadas
(Integrante 1-4), una por estudiante del grupo. Se reordenan/ajustan los
criterios: Trabajan en clases (antes 2°, ahora 1°), Todos los integrantes
participan (reemplaza "Trabaja en equipo" con una redacción más
observable), Presenta dudas y Hace entrega de su trabajo se mantienen, y
se agrega un quinto criterio: Análisis de datos. Las 5 columnas de
criterios mantienen el desplegable Sí/No.
</commit_message>
<xml_diff>
--- a/portafolio-docente-2026/lista-cotejo-investigacion-grupal.xlsx
+++ b/portafolio-docente-2026/lista-cotejo-investigacion-grupal.xlsx
@@ -104,7 +104,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -128,9 +128,6 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -138,9 +135,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -253,7 +247,7 @@
   </oneCellAnchor>
   <oneCellAnchor>
     <from>
-      <col>5</col>
+      <col>10</col>
       <colOff>0</colOff>
       <row>0</row>
       <rowOff>0</rowOff>
@@ -568,33 +562,36 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G16"/>
+  <dimension ref="A1:K16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="16" customWidth="1" min="2" max="2"/>
-    <col width="32" customWidth="1" min="3" max="3"/>
-    <col width="16" customWidth="1" min="4" max="4"/>
-    <col width="16" customWidth="1" min="5" max="5"/>
-    <col width="16" customWidth="1" min="6" max="6"/>
-    <col width="20" customWidth="1" min="7" max="7"/>
+    <col width="24" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="18" customWidth="1" min="10" max="10"/>
+    <col width="16" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
-      <c r="C1" s="1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Colegio Presidente José Joaquín Prieto</t>
         </is>
       </c>
     </row>
     <row r="2" ht="18" customHeight="1">
-      <c r="C2" s="2" t="inlineStr">
+      <c r="D2" s="2" t="inlineStr">
         <is>
           <t>Red de Colegios SIP</t>
         </is>
       </c>
     </row>
-    <row r="3" ht="14" customHeight="1"/>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
@@ -609,7 +606,7 @@
         </is>
       </c>
     </row>
-    <row r="8" ht="32" customHeight="1">
+    <row r="8" ht="34" customHeight="1">
       <c r="A8" s="5" t="inlineStr">
         <is>
           <t>Grupo</t>
@@ -622,31 +619,51 @@
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>Integrantes</t>
+          <t>Integrante 1</t>
         </is>
       </c>
       <c r="D8" s="5" t="inlineStr">
         <is>
-          <t>Trabaja en equipo</t>
+          <t>Integrante 2</t>
         </is>
       </c>
       <c r="E8" s="5" t="inlineStr">
         <is>
-          <t>Trabaja en clases</t>
+          <t>Integrante 3</t>
         </is>
       </c>
       <c r="F8" s="5" t="inlineStr">
         <is>
+          <t>Integrante 4</t>
+        </is>
+      </c>
+      <c r="G8" s="5" t="inlineStr">
+        <is>
+          <t>Trabajan en clases</t>
+        </is>
+      </c>
+      <c r="H8" s="5" t="inlineStr">
+        <is>
+          <t>Todos los integrantes participan</t>
+        </is>
+      </c>
+      <c r="I8" s="5" t="inlineStr">
+        <is>
           <t>Presenta dudas</t>
         </is>
       </c>
-      <c r="G8" s="5" t="inlineStr">
+      <c r="J8" s="5" t="inlineStr">
         <is>
           <t>Hace entrega de su trabajo</t>
         </is>
       </c>
-    </row>
-    <row r="9" ht="42" customHeight="1">
+      <c r="K8" s="5" t="inlineStr">
+        <is>
+          <t>Análisis de datos</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="30" customHeight="1">
       <c r="A9" s="6" t="inlineStr">
         <is>
           <t>GRUPO N°1</t>
@@ -658,29 +675,37 @@
         </is>
       </c>
       <c r="C9" s="8" t="inlineStr"/>
-      <c r="D9" s="9" t="inlineStr"/>
-      <c r="E9" s="9" t="inlineStr"/>
-      <c r="F9" s="9" t="inlineStr"/>
-      <c r="G9" s="9" t="inlineStr"/>
-    </row>
-    <row r="10" ht="42" customHeight="1">
-      <c r="A10" s="10" t="inlineStr">
+      <c r="D9" s="8" t="inlineStr"/>
+      <c r="E9" s="8" t="inlineStr"/>
+      <c r="F9" s="8" t="inlineStr"/>
+      <c r="G9" s="8" t="inlineStr"/>
+      <c r="H9" s="8" t="inlineStr"/>
+      <c r="I9" s="8" t="inlineStr"/>
+      <c r="J9" s="8" t="inlineStr"/>
+      <c r="K9" s="8" t="inlineStr"/>
+    </row>
+    <row r="10" ht="30" customHeight="1">
+      <c r="A10" s="9" t="inlineStr">
         <is>
           <t>GRUPO N°2</t>
         </is>
       </c>
-      <c r="B10" s="11" t="inlineStr">
+      <c r="B10" s="10" t="inlineStr">
         <is>
           <t>Recopiladora folclórica</t>
         </is>
       </c>
-      <c r="C10" s="12" t="inlineStr"/>
-      <c r="D10" s="13" t="inlineStr"/>
-      <c r="E10" s="13" t="inlineStr"/>
-      <c r="F10" s="13" t="inlineStr"/>
-      <c r="G10" s="13" t="inlineStr"/>
-    </row>
-    <row r="11" ht="42" customHeight="1">
+      <c r="C10" s="11" t="inlineStr"/>
+      <c r="D10" s="11" t="inlineStr"/>
+      <c r="E10" s="11" t="inlineStr"/>
+      <c r="F10" s="11" t="inlineStr"/>
+      <c r="G10" s="11" t="inlineStr"/>
+      <c r="H10" s="11" t="inlineStr"/>
+      <c r="I10" s="11" t="inlineStr"/>
+      <c r="J10" s="11" t="inlineStr"/>
+      <c r="K10" s="11" t="inlineStr"/>
+    </row>
+    <row r="11" ht="30" customHeight="1">
       <c r="A11" s="6" t="inlineStr">
         <is>
           <t>GRUPO N°3</t>
@@ -692,29 +717,37 @@
         </is>
       </c>
       <c r="C11" s="8" t="inlineStr"/>
-      <c r="D11" s="9" t="inlineStr"/>
-      <c r="E11" s="9" t="inlineStr"/>
-      <c r="F11" s="9" t="inlineStr"/>
-      <c r="G11" s="9" t="inlineStr"/>
-    </row>
-    <row r="12" ht="42" customHeight="1">
-      <c r="A12" s="10" t="inlineStr">
+      <c r="D11" s="8" t="inlineStr"/>
+      <c r="E11" s="8" t="inlineStr"/>
+      <c r="F11" s="8" t="inlineStr"/>
+      <c r="G11" s="8" t="inlineStr"/>
+      <c r="H11" s="8" t="inlineStr"/>
+      <c r="I11" s="8" t="inlineStr"/>
+      <c r="J11" s="8" t="inlineStr"/>
+      <c r="K11" s="8" t="inlineStr"/>
+    </row>
+    <row r="12" ht="30" customHeight="1">
+      <c r="A12" s="9" t="inlineStr">
         <is>
           <t>GRUPO N°4</t>
         </is>
       </c>
-      <c r="B12" s="11" t="inlineStr">
+      <c r="B12" s="10" t="inlineStr">
         <is>
           <t>Nacimiento y familia</t>
         </is>
       </c>
-      <c r="C12" s="12" t="inlineStr"/>
-      <c r="D12" s="13" t="inlineStr"/>
-      <c r="E12" s="13" t="inlineStr"/>
-      <c r="F12" s="13" t="inlineStr"/>
-      <c r="G12" s="13" t="inlineStr"/>
-    </row>
-    <row r="13" ht="42" customHeight="1">
+      <c r="C12" s="11" t="inlineStr"/>
+      <c r="D12" s="11" t="inlineStr"/>
+      <c r="E12" s="11" t="inlineStr"/>
+      <c r="F12" s="11" t="inlineStr"/>
+      <c r="G12" s="11" t="inlineStr"/>
+      <c r="H12" s="11" t="inlineStr"/>
+      <c r="I12" s="11" t="inlineStr"/>
+      <c r="J12" s="11" t="inlineStr"/>
+      <c r="K12" s="11" t="inlineStr"/>
+    </row>
+    <row r="13" ht="30" customHeight="1">
       <c r="A13" s="6" t="inlineStr">
         <is>
           <t>GRUPO N°5</t>
@@ -726,30 +759,38 @@
         </is>
       </c>
       <c r="C13" s="8" t="inlineStr"/>
-      <c r="D13" s="9" t="inlineStr"/>
-      <c r="E13" s="9" t="inlineStr"/>
-      <c r="F13" s="9" t="inlineStr"/>
-      <c r="G13" s="9" t="inlineStr"/>
-    </row>
-    <row r="14" ht="42" customHeight="1">
-      <c r="A14" s="10" t="inlineStr">
+      <c r="D13" s="8" t="inlineStr"/>
+      <c r="E13" s="8" t="inlineStr"/>
+      <c r="F13" s="8" t="inlineStr"/>
+      <c r="G13" s="8" t="inlineStr"/>
+      <c r="H13" s="8" t="inlineStr"/>
+      <c r="I13" s="8" t="inlineStr"/>
+      <c r="J13" s="8" t="inlineStr"/>
+      <c r="K13" s="8" t="inlineStr"/>
+    </row>
+    <row r="14" ht="30" customHeight="1">
+      <c r="A14" s="9" t="inlineStr">
         <is>
           <t>GRUPO N°6</t>
         </is>
       </c>
-      <c r="B14" s="11" t="inlineStr">
+      <c r="B14" s="10" t="inlineStr">
         <is>
           <t>Artista visual y Louvre</t>
         </is>
       </c>
-      <c r="C14" s="12" t="inlineStr"/>
-      <c r="D14" s="13" t="inlineStr"/>
-      <c r="E14" s="13" t="inlineStr"/>
-      <c r="F14" s="13" t="inlineStr"/>
-      <c r="G14" s="13" t="inlineStr"/>
+      <c r="C14" s="11" t="inlineStr"/>
+      <c r="D14" s="11" t="inlineStr"/>
+      <c r="E14" s="11" t="inlineStr"/>
+      <c r="F14" s="11" t="inlineStr"/>
+      <c r="G14" s="11" t="inlineStr"/>
+      <c r="H14" s="11" t="inlineStr"/>
+      <c r="I14" s="11" t="inlineStr"/>
+      <c r="J14" s="11" t="inlineStr"/>
+      <c r="K14" s="11" t="inlineStr"/>
     </row>
     <row r="16">
-      <c r="A16" s="14" t="inlineStr">
+      <c r="A16" s="12" t="inlineStr">
         <is>
           <t>Marca Sí/No en cada criterio (usa el menú desplegable). Esta lista mide solo el trabajo de investigación grupal, no la participación individual en mano alzada/gira y discute.</t>
         </is>
@@ -757,14 +798,14 @@
     </row>
   </sheetData>
   <mergeCells count="5">
-    <mergeCell ref="C2:E2"/>
-    <mergeCell ref="C1:E1"/>
-    <mergeCell ref="A6:G6"/>
-    <mergeCell ref="A16:G16"/>
-    <mergeCell ref="A5:G5"/>
+    <mergeCell ref="A6:K6"/>
+    <mergeCell ref="D2:H2"/>
+    <mergeCell ref="D1:H1"/>
+    <mergeCell ref="A16:K16"/>
+    <mergeCell ref="A5:K5"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation sqref="D9:G14" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="G9:G14 H9:H14 I9:I14 J9:J14 K9:K14" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Sí,No"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Separar el análisis de datos del criterio de evaluación y agregar desplegable en Temática
Se corrige un malentendido: "análisis de datos" no es algo que se le pida
a los estudiantes (no era un criterio más de la lista de cotejo), sino un
resumen que el propio profesor necesita a partir de lo que marque. Se
quita esa columna y se agrega, debajo de la tabla, una sección de
"Análisis de datos" con fórmulas COUNTIF que calculan automáticamente,
por cada uno de los 4 criterios reales, cuántos grupos obtuvieron Sí/No
y el % de cumplimiento sobre los 6 grupos. Se agrega también un menú
desplegable en la columna "Temática asignada" (las 3 temáticas de
investigación), que antes era texto fijo.
</commit_message>
<xml_diff>
--- a/portafolio-docente-2026/lista-cotejo-investigacion-grupal.xlsx
+++ b/portafolio-docente-2026/lista-cotejo-investigacion-grupal.xlsx
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="7">
+  <fonts count="8">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -54,8 +54,13 @@
       <color rgb="00555555"/>
       <sz val="9"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="001F3864"/>
+      <sz val="12"/>
+    </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -75,6 +80,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00F2F4F8"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="002E75B6"/>
       </patternFill>
     </fill>
   </fills>
@@ -104,7 +114,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -141,6 +151,21 @@
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -247,7 +272,7 @@
   </oneCellAnchor>
   <oneCellAnchor>
     <from>
-      <col>10</col>
+      <col>9</col>
       <colOff>0</colOff>
       <row>0</row>
       <rowOff>0</rowOff>
@@ -562,7 +587,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K16"/>
+  <dimension ref="A1:J25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -572,10 +597,9 @@
     <col width="18" customWidth="1" min="5" max="5"/>
     <col width="18" customWidth="1" min="6" max="6"/>
     <col width="16" customWidth="1" min="7" max="7"/>
-    <col width="18" customWidth="1" min="8" max="8"/>
+    <col width="20" customWidth="1" min="8" max="8"/>
     <col width="14" customWidth="1" min="9" max="9"/>
-    <col width="18" customWidth="1" min="10" max="10"/>
-    <col width="16" customWidth="1" min="11" max="11"/>
+    <col width="20" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
@@ -655,11 +679,6 @@
       <c r="J8" s="5" t="inlineStr">
         <is>
           <t>Hace entrega de su trabajo</t>
-        </is>
-      </c>
-      <c r="K8" s="5" t="inlineStr">
-        <is>
-          <t>Análisis de datos</t>
         </is>
       </c>
     </row>
@@ -682,7 +701,6 @@
       <c r="H9" s="8" t="inlineStr"/>
       <c r="I9" s="8" t="inlineStr"/>
       <c r="J9" s="8" t="inlineStr"/>
-      <c r="K9" s="8" t="inlineStr"/>
     </row>
     <row r="10" ht="30" customHeight="1">
       <c r="A10" s="9" t="inlineStr">
@@ -703,7 +721,6 @@
       <c r="H10" s="11" t="inlineStr"/>
       <c r="I10" s="11" t="inlineStr"/>
       <c r="J10" s="11" t="inlineStr"/>
-      <c r="K10" s="11" t="inlineStr"/>
     </row>
     <row r="11" ht="30" customHeight="1">
       <c r="A11" s="6" t="inlineStr">
@@ -724,7 +741,6 @@
       <c r="H11" s="8" t="inlineStr"/>
       <c r="I11" s="8" t="inlineStr"/>
       <c r="J11" s="8" t="inlineStr"/>
-      <c r="K11" s="8" t="inlineStr"/>
     </row>
     <row r="12" ht="30" customHeight="1">
       <c r="A12" s="9" t="inlineStr">
@@ -745,7 +761,6 @@
       <c r="H12" s="11" t="inlineStr"/>
       <c r="I12" s="11" t="inlineStr"/>
       <c r="J12" s="11" t="inlineStr"/>
-      <c r="K12" s="11" t="inlineStr"/>
     </row>
     <row r="13" ht="30" customHeight="1">
       <c r="A13" s="6" t="inlineStr">
@@ -766,7 +781,6 @@
       <c r="H13" s="8" t="inlineStr"/>
       <c r="I13" s="8" t="inlineStr"/>
       <c r="J13" s="8" t="inlineStr"/>
-      <c r="K13" s="8" t="inlineStr"/>
     </row>
     <row r="14" ht="30" customHeight="1">
       <c r="A14" s="9" t="inlineStr">
@@ -787,7 +801,6 @@
       <c r="H14" s="11" t="inlineStr"/>
       <c r="I14" s="11" t="inlineStr"/>
       <c r="J14" s="11" t="inlineStr"/>
-      <c r="K14" s="11" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="12" t="inlineStr">
@@ -796,17 +809,134 @@
         </is>
       </c>
     </row>
+    <row r="18">
+      <c r="A18" s="13" t="inlineStr">
+        <is>
+          <t>Análisis de datos (se calcula automáticamente con lo que marques arriba)</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="14" t="inlineStr">
+        <is>
+          <t>Criterio</t>
+        </is>
+      </c>
+      <c r="B19" s="14" t="inlineStr">
+        <is>
+          <t>N° de grupos con Sí</t>
+        </is>
+      </c>
+      <c r="C19" s="14" t="inlineStr">
+        <is>
+          <t>N° de grupos con No</t>
+        </is>
+      </c>
+      <c r="D19" s="14" t="inlineStr">
+        <is>
+          <t>% de cumplimiento</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="15" t="inlineStr">
+        <is>
+          <t>Trabajan en clases</t>
+        </is>
+      </c>
+      <c r="B20" s="16">
+        <f>COUNTIF(G9:G14,"Sí")</f>
+        <v/>
+      </c>
+      <c r="C20" s="16">
+        <f>COUNTIF(G9:G14,"No")</f>
+        <v/>
+      </c>
+      <c r="D20" s="17">
+        <f>COUNTIF(G9:G14,"Sí")/6</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="15" t="inlineStr">
+        <is>
+          <t>Todos los integrantes participan</t>
+        </is>
+      </c>
+      <c r="B21" s="16">
+        <f>COUNTIF(H9:H14,"Sí")</f>
+        <v/>
+      </c>
+      <c r="C21" s="16">
+        <f>COUNTIF(H9:H14,"No")</f>
+        <v/>
+      </c>
+      <c r="D21" s="17">
+        <f>COUNTIF(H9:H14,"Sí")/6</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="15" t="inlineStr">
+        <is>
+          <t>Presenta dudas</t>
+        </is>
+      </c>
+      <c r="B22" s="16">
+        <f>COUNTIF(I9:I14,"Sí")</f>
+        <v/>
+      </c>
+      <c r="C22" s="16">
+        <f>COUNTIF(I9:I14,"No")</f>
+        <v/>
+      </c>
+      <c r="D22" s="17">
+        <f>COUNTIF(I9:I14,"Sí")/6</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="15" t="inlineStr">
+        <is>
+          <t>Hace entrega de su trabajo</t>
+        </is>
+      </c>
+      <c r="B23" s="16">
+        <f>COUNTIF(J9:J14,"Sí")</f>
+        <v/>
+      </c>
+      <c r="C23" s="16">
+        <f>COUNTIF(J9:J14,"No")</f>
+        <v/>
+      </c>
+      <c r="D23" s="17">
+        <f>COUNTIF(J9:J14,"Sí")/6</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="12" t="inlineStr">
+        <is>
+          <t>El % de cumplimiento se calcula sobre los 6 grupos. Estos datos sirven como evidencia cuantitativa del trabajo de investigación grupal de la Clase 1.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="5">
-    <mergeCell ref="A6:K6"/>
+  <mergeCells count="7">
+    <mergeCell ref="A5:J5"/>
+    <mergeCell ref="A6:J6"/>
     <mergeCell ref="D2:H2"/>
+    <mergeCell ref="A18:J18"/>
     <mergeCell ref="D1:H1"/>
-    <mergeCell ref="A16:K16"/>
-    <mergeCell ref="A5:K5"/>
+    <mergeCell ref="A16:J16"/>
+    <mergeCell ref="A25:J25"/>
   </mergeCells>
-  <dataValidations count="1">
-    <dataValidation sqref="G9:G14 H9:H14 I9:I14 J9:J14 K9:K14" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+  <dataValidations count="2">
+    <dataValidation sqref="G9:G14 H9:H14 I9:I14 J9:J14" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Sí,No"</formula1>
+    </dataValidation>
+    <dataValidation sqref="B9:B14" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Nacimiento y familia,Recopiladora folclórica,Artista visual y Louvre"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>